<commit_message>
Revisión ampliada, vuelta 3: tildes del Gantt, valores de la lista de componentes
- Gantt (por el Google Sheet): «biometría», «Dólar», «Acá», «Inversión» y un espacio de más;
  bajado otra vez del Drive.
- Lista de componentes: las fórmulas guardan su valor (en un visor los subtotales salían vacíos).
- Registro de la vuelta 3 en CAMBIOS_REVISION.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QiY8ZZNAM9gwPKiqSkCaaj
</commit_message>
<xml_diff>
--- a/documentacion_proyecto/Lista_de_componentes_Control_Trama.xlsx
+++ b/documentacion_proyecto/Lista_de_componentes_Control_Trama.xlsx
@@ -1211,7 +1211,7 @@
       </c>
       <c r="E6" s="72">
         <f>C6*D6</f>
-        <v/>
+        <v>12203</v>
       </c>
       <c r="F6" s="123" t="inlineStr">
         <is>
@@ -1243,7 +1243,7 @@
       </c>
       <c r="E7" s="72">
         <f>C7*D7</f>
-        <v/>
+        <v>5000</v>
       </c>
       <c r="F7" s="123" t="inlineStr">
         <is>
@@ -1275,7 +1275,7 @@
       </c>
       <c r="E8" s="72">
         <f>C8*D8</f>
-        <v/>
+        <v>7000</v>
       </c>
       <c r="F8" s="80" t="inlineStr">
         <is>
@@ -1307,7 +1307,7 @@
       </c>
       <c r="E9" s="72">
         <f>C9*D9</f>
-        <v/>
+        <v>1500</v>
       </c>
       <c r="F9" s="80" t="inlineStr">
         <is>
@@ -1339,7 +1339,7 @@
       </c>
       <c r="E10" s="72">
         <f>C10*D10</f>
-        <v/>
+        <v>1500</v>
       </c>
       <c r="F10" s="80" t="inlineStr">
         <is>
@@ -1371,7 +1371,7 @@
       </c>
       <c r="E11" s="127">
         <f>C11*D11</f>
-        <v/>
+        <v>450</v>
       </c>
       <c r="F11" s="80" t="inlineStr">
         <is>
@@ -1403,7 +1403,7 @@
       </c>
       <c r="E12" s="72">
         <f>C12*D12</f>
-        <v/>
+        <v>900</v>
       </c>
       <c r="F12" s="80" t="inlineStr">
         <is>
@@ -1435,7 +1435,7 @@
       </c>
       <c r="E13" s="72">
         <f>C13*D13</f>
-        <v/>
+        <v>900</v>
       </c>
       <c r="F13" s="80" t="inlineStr">
         <is>
@@ -1467,7 +1467,7 @@
       </c>
       <c r="E14" s="72">
         <f>C14*D14</f>
-        <v/>
+        <v>300</v>
       </c>
       <c r="F14" s="80" t="inlineStr">
         <is>
@@ -1499,7 +1499,7 @@
       </c>
       <c r="E15" s="72">
         <f>C15*D15</f>
-        <v/>
+        <v>15000</v>
       </c>
       <c r="F15" s="123" t="inlineStr">
         <is>
@@ -1531,7 +1531,7 @@
       </c>
       <c r="E16" s="72">
         <f>C16*D16</f>
-        <v/>
+        <v>16000</v>
       </c>
       <c r="F16" s="80" t="inlineStr">
         <is>
@@ -1563,7 +1563,7 @@
       </c>
       <c r="E17" s="72">
         <f>C17*D17</f>
-        <v/>
+        <v>3200</v>
       </c>
       <c r="F17" s="80" t="inlineStr">
         <is>
@@ -1595,7 +1595,7 @@
       </c>
       <c r="E18" s="72">
         <f>C18*D18</f>
-        <v/>
+        <v>1000</v>
       </c>
       <c r="F18" s="80" t="inlineStr">
         <is>
@@ -1627,7 +1627,7 @@
       </c>
       <c r="E19" s="72">
         <f>C19*D19</f>
-        <v/>
+        <v>7500</v>
       </c>
       <c r="F19" s="80" t="inlineStr">
         <is>
@@ -1659,7 +1659,7 @@
       </c>
       <c r="E20" s="72">
         <f>C20*D20</f>
-        <v/>
+        <v>1200</v>
       </c>
       <c r="F20" s="80" t="inlineStr">
         <is>
@@ -1683,7 +1683,7 @@
       <c r="D21" s="88" t="n"/>
       <c r="E21" s="89">
         <f>SUM(E6:E20)</f>
-        <v/>
+        <v>73653</v>
       </c>
       <c r="F21" s="90" t="n"/>
       <c r="G21" s="91" t="n"/>
@@ -1758,7 +1758,7 @@
       </c>
       <c r="E25" s="72">
         <f>C25*D25</f>
-        <v/>
+        <v>7000</v>
       </c>
       <c r="F25" s="98" t="inlineStr">
         <is>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="E26" s="72">
         <f>C26*D26</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F26" s="98" t="inlineStr">
         <is>
@@ -1822,7 +1822,7 @@
       </c>
       <c r="E27" s="72">
         <f>C27*D27</f>
-        <v/>
+        <v>1400</v>
       </c>
       <c r="F27" s="98" t="inlineStr">
         <is>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="E28" s="72">
         <f>C28*D28</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F28" s="98" t="inlineStr">
         <is>
@@ -1886,7 +1886,7 @@
       </c>
       <c r="E29" s="72">
         <f>C29*D29</f>
-        <v/>
+        <v>5100</v>
       </c>
       <c r="F29" s="98" t="inlineStr">
         <is>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="E30" s="72">
         <f>C30*D30</f>
-        <v/>
+        <v>300</v>
       </c>
       <c r="F30" s="98" t="inlineStr">
         <is>
@@ -1950,7 +1950,7 @@
       </c>
       <c r="E31" s="72">
         <f>C31*D31</f>
-        <v/>
+        <v>150</v>
       </c>
       <c r="F31" s="98" t="inlineStr">
         <is>
@@ -1982,7 +1982,7 @@
       </c>
       <c r="E32" s="72">
         <f>C32*D32</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F32" s="98" t="inlineStr">
         <is>
@@ -2014,7 +2014,7 @@
       </c>
       <c r="E33" s="72">
         <f>C33*D33</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F33" s="98" t="inlineStr">
         <is>
@@ -2038,7 +2038,7 @@
       <c r="D34" s="88" t="n"/>
       <c r="E34" s="103">
         <f>SUM(E25:E33)</f>
-        <v/>
+        <v>13950</v>
       </c>
       <c r="F34" s="104" t="n"/>
       <c r="G34" s="90" t="n"/>
@@ -2113,7 +2113,7 @@
       </c>
       <c r="E38" s="72">
         <f>C38*D38</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F38" s="98" t="inlineStr">
         <is>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="E39" s="72">
         <f>C39*D39</f>
-        <v/>
+        <v>24136</v>
       </c>
       <c r="F39" s="98" t="inlineStr">
         <is>
@@ -2177,7 +2177,7 @@
       </c>
       <c r="E40" s="110">
         <f>C40*D40</f>
-        <v/>
+        <v>3600</v>
       </c>
       <c r="F40" s="98" t="inlineStr">
         <is>
@@ -2209,7 +2209,7 @@
       </c>
       <c r="E41" s="72">
         <f>C41*D41</f>
-        <v/>
+        <v>5600</v>
       </c>
       <c r="F41" s="98" t="inlineStr">
         <is>
@@ -2241,7 +2241,7 @@
       </c>
       <c r="E42" s="72">
         <f>C42*D42</f>
-        <v/>
+        <v>600</v>
       </c>
       <c r="F42" s="98" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
       </c>
       <c r="E43" s="110">
         <f>C43*D43</f>
-        <v/>
+        <v>600</v>
       </c>
       <c r="F43" s="98" t="inlineStr">
         <is>
@@ -2303,7 +2303,7 @@
       <c r="D44" s="71" t="n"/>
       <c r="E44" s="72">
         <f>C44*D44</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F44" s="98" t="inlineStr">
         <is>
@@ -2333,7 +2333,7 @@
       <c r="D45" s="71" t="n"/>
       <c r="E45" s="72">
         <f>C45*D45</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F45" s="98" t="inlineStr">
         <is>
@@ -2363,7 +2363,7 @@
       <c r="D46" s="71" t="n"/>
       <c r="E46" s="72">
         <f>C46*D46</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F46" s="98" t="inlineStr">
         <is>
@@ -2393,7 +2393,7 @@
       <c r="D47" s="71" t="n"/>
       <c r="E47" s="72">
         <f>C47*D47</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F47" s="98" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
       <c r="D48" s="71" t="n"/>
       <c r="E48" s="72">
         <f>C48*D48</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F48" s="98" t="inlineStr">
         <is>
@@ -2453,7 +2453,7 @@
       <c r="D49" s="71" t="n"/>
       <c r="E49" s="72">
         <f>C49*D49</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F49" s="98" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       <c r="D50" s="71" t="n"/>
       <c r="E50" s="72">
         <f>C50*D50</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F50" s="98" t="inlineStr">
         <is>
@@ -2513,7 +2513,7 @@
       <c r="D51" s="71" t="n"/>
       <c r="E51" s="72">
         <f>C51*D51</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F51" s="98" t="inlineStr">
         <is>
@@ -2543,7 +2543,7 @@
       <c r="D52" s="71" t="n"/>
       <c r="E52" s="72">
         <f>C52*D52</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="F52" s="98" t="inlineStr">
         <is>
@@ -2567,7 +2567,7 @@
       <c r="D53" s="88" t="n"/>
       <c r="E53" s="113">
         <f>SUM(E38:E52)</f>
-        <v/>
+        <v>34536</v>
       </c>
       <c r="F53" s="114" t="n"/>
       <c r="G53" s="115" t="n"/>
@@ -2584,7 +2584,7 @@
       <c r="D55" s="118" t="n"/>
       <c r="E55" s="119">
         <f>E21+E34+E53</f>
-        <v/>
+        <v>122139</v>
       </c>
       <c r="F55" s="120" t="n"/>
       <c r="G55" s="121" t="n"/>

</xml_diff>

<commit_message>
Las cinco plaquetas soldadas, terminadas, en toda la documentación
La tarea 7,2 del Gantt está al 100 %: los Word (Documentación de Proyecto, Estado, Bitácora,
Árbol, Guía de los relés, Manual del telar, Parado automático), sus PDF, la Lista de componentes
y los Markdown ya no dan las plaquetas como pendientes. Quedan el gabinete en la planta y los
otros tres canales.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QiY8ZZNAM9gwPKiqSkCaaj
</commit_message>
<xml_diff>
--- a/documentacion_proyecto/Lista_de_componentes_Control_Trama.xlsx
+++ b/documentacion_proyecto/Lista_de_componentes_Control_Trama.xlsx
@@ -2312,7 +2312,7 @@
       </c>
       <c r="G44" s="74" t="inlineStr">
         <is>
-          <t>Se suma el 10/10/2026: con todo probado en protoboard, se está haciendo la plaqueta para probar todo de manera correcta. Precio a completar.</t>
+          <t>Se suma el 10/10/2026, con todo probado en protoboard. Ya está soldada (20/10/2026). Precio a completar.</t>
         </is>
       </c>
     </row>
@@ -2593,7 +2593,7 @@
     <row r="57" ht="21.75" customHeight="1" s="59">
       <c r="A57" s="122" t="inlineStr">
         <is>
-          <t>• ORDEN DE COMPRA: (1) Bloque A: comprado e instalado en el telar (19/09/2026). (2) Medición de la alimentación y la señal de un lector óptico: hecha el 17/10/2026, entre 15 y 30 V (la velocidad ya está confirmada: 300 pasadas por minuto). (3) Recién entonces el Bloque D, con la conexión final: el relé en lugar del lector, con una resistencia de protección que se elige con esa medición. Estado al 17/10/2026: el Nivel 2 (sensor de pasada y relé LCA110) se probó en protoboard el 10/10/2026 y en el telar el 17/10/2026, con el sensor y el primer canal: funcionó; se están haciendo las plaquetas para la instalación definitiva.</t>
+          <t>• ORDEN DE COMPRA: (1) Bloque A: comprado e instalado en el telar (19/09/2026). (2) Medición de la alimentación y la señal de un lector óptico: hecha el 17/10/2026, entre 15 y 30 V (la velocidad ya está confirmada: 300 pasadas por minuto). (3) Recién entonces el Bloque D, con la conexión final: el relé en lugar del lector, con una resistencia de protección que se elige con esa medición. Estado al 20/10/2026: el Nivel 2 (sensor de pasada y relé LCA110) se probó en protoboard el 10/10/2026 y en el telar el 17/10/2026, con el sensor y el primer canal: funcionó, y al 20/10/2026 las plaquetas para la instalación definitiva ya están soldadas.</t>
         </is>
       </c>
     </row>

</xml_diff>